<commit_message>
Correct dashboard totals, align 12 gap areas, and clean PDF footers
</commit_message>
<xml_diff>
--- a/PeachtreePay_ISO27001_GRC_Portfolio.xlsx
+++ b/PeachtreePay_ISO27001_GRC_Portfolio.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R16347d1adf18419e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="2" r:id="R8ff923b63db54e9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Treatment Plan" sheetId="3" r:id="R5a43c99b8800423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Assessment" sheetId="4" r:id="R3b9e1e3be0f94704"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statement of Applicability" sheetId="5" r:id="R590ae7feedf649c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="6" r:id="Rc125763acbda41a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R01420edec4b24e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Register" sheetId="2" r:id="R38a89a1833794166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Treatment Plan" sheetId="3" r:id="Rfc23f07452624b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Assessment" sheetId="4" r:id="R05c301552ff84f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statement of Applicability" sheetId="5" r:id="Rf6596f3f41254213"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Register" sheetId="6" r:id="Ree8903682a874dfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -143,28 +143,28 @@
         <x:b/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF4CCCC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE5CD"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9EAD3"/>
         </x:patternFill>
       </x:fill>
@@ -405,6 +405,7 @@
         <x:v>Total Risks</x:v>
       </x:c>
       <x:c r="B4" s="20" t="n">
+        <x:f>COUNT('Risk Register'!A2:A16)</x:f>
         <x:v>15</x:v>
       </x:c>
       <x:c r="D4" s="20" t="str">
@@ -419,6 +420,7 @@
         <x:v>Critical Inherent Risks</x:v>
       </x:c>
       <x:c r="B5" s="20" t="n">
+        <x:f>COUNTIF('Risk Register'!G2:G16,"Critical")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D5" s="20" t="str">
@@ -433,7 +435,8 @@
         <x:v>High Inherent Risks</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Risk Register'!G2:G16,"High")</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="20" t="str">
         <x:v>Gap Assessment</x:v>
@@ -447,6 +450,7 @@
         <x:v>Gap Areas Reviewed</x:v>
       </x:c>
       <x:c r="B7" s="20" t="n">
+        <x:f>COUNTA('Gap Assessment'!A2:A13)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D7" s="20" t="str">

</xml_diff>